<commit_message>
adapte el  código para que los archivos se guarden en las carpetas correspondientes
</commit_message>
<xml_diff>
--- a/visualizations/reporte_ADO_hallazgos.xlsx
+++ b/visualizations/reporte_ADO_hallazgos.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>97.8</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>98</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>99</v>
+        <v>99.2</v>
       </c>
     </row>
     <row r="15">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>98.59999999999999</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="33">
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>98.7</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="39">
@@ -1639,11 +1639,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="82">
@@ -1654,11 +1654,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>95.8</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
     <row r="83">
@@ -1669,11 +1669,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>94.40000000000001</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="84">
@@ -1684,11 +1684,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>97.2</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="85">
@@ -1699,11 +1699,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>95.8</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="86">
@@ -1714,11 +1714,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>97.09999999999999</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="87">
@@ -1729,11 +1729,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>99.59999999999999</v>
+        <v>97.09999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -1744,11 +1744,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>96.09999999999999</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="89">
@@ -1759,11 +1759,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>95.40000000000001</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="90">
@@ -1774,11 +1774,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>95.8</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="91">
@@ -1789,10 +1789,25 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>95.8</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>CDMX-TOLUCA</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C91" t="n">
+      <c r="C92" t="n">
         <v>94.5</v>
       </c>
     </row>
@@ -2214,7 +2229,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>49.6</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="28">
@@ -2409,7 +2424,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>58.1</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="41">
@@ -3189,7 +3204,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>58.7</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="93">
@@ -3234,7 +3249,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>51.2</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="96">

</xml_diff>